<commit_message>
Thêm GlobalExceptionHandler, các trang lỗi và thêm trạng thái để làm tính năng đăng ký thi đấu
</commit_message>
<xml_diff>
--- a/Jame exercises of module 4_final.xlsx
+++ b/Jame exercises of module 4_final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CODEGYM\bai_tap_code_gym\module_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F5ABF5-9F9D-4BFF-AFCA-27064C7168E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97774855-817D-46B5-A260-E004C420C66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Tổng quan Spring MVC" sheetId="1" r:id="rId1"/>
@@ -155,12 +155,188 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
+    <t xml:space="preserve">Bài 1: Nâng cấp ứng dụng quản lý cầu thủ bóng đá </t>
+  </si>
+  <si>
+    <t>Ngoài các chức năng hiện có, ứng dụng còn cho phép tạo đội hình 11 người dựa trên danh sách cầu thủ hiện tại.</t>
+  </si>
+  <si>
+    <t>Ở màn hình danh sách cầu thủ, mặc định trạng thái của một cầu thủ là "Dự bị".</t>
+  </si>
+  <si>
+    <t>Mỗi lần cầu thủ được [Đăng ký đá] thì trạng thái cầu thủ sẽ thay đổi "Đã đăng ký".</t>
+  </si>
+  <si>
+    <t>Một cầu thủ có thể bị huỷ đăng ký, thì trạng thái sẽ được chuyển lại thành "Dự bị".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số lượng cầu thủ đăng ký tối đã chỉ được phép là 11 người. </t>
+  </si>
+  <si>
+    <t>Thực hiện 3 chức năng sau:</t>
+  </si>
+  <si>
+    <t>1. Nếu số lượng cầu thủ đăng ký vượt quá 11 thì sẽ chuyển sang màn hình lỗi.</t>
+  </si>
+  <si>
+    <t>2. Thực hiện ghi log tất cả các hành động khiến trạng thái cầu thủ bị thay đổi.</t>
+  </si>
+  <si>
+    <t>- "Dự bị" -&gt; "Đăng ký đá".</t>
+  </si>
+  <si>
+    <t>- "Đăng ký đá" -&gt; "Dự bị".</t>
+  </si>
+  <si>
+    <t>3. Thực hiện ghi log số lượng cầu thủ được đăng ký đá.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Times New Roman"/>
       </rPr>
+      <t xml:space="preserve">Bước 1: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t>Chỉnh sửa màn hình danh sách cầu thủ, chuyển đổi từ table sang dạng card, như bên dưới:</t>
+    </r>
+  </si>
+  <si>
+    <t>https://getbootstrap.com/docs/5.3/components/card/#example</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t xml:space="preserve">Bước 2: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t>Khi người dùng click vào cầu thủ bất kì, sẽ chuyển tiếp đến trang Chi tiết cầu thủ.</t>
+    </r>
+  </si>
+  <si>
+    <t>Khi click vào button [Yêu thích], thì cầu thủ sẽ được cập nhật vào danh sách yêu thích.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t>Lưu ý</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t>: Lưu trữ danh sách cầu thủ yêu thích vào Session.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t>Bước 3:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t xml:space="preserve"> Khi vào màn hình Danh sách cầu thủ yêu thích, thì sẽ hiển thị toàn bộ cầu thủ đã được Yêu thích ở Bước 2.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t xml:space="preserve">Bước 4: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t>Ngoài ra, cần giữ lại danh sách yêu thích khi tắt browser, sử dụng Cookie để thực hiện việc này.</t>
+    </r>
+  </si>
+  <si>
+    <t>Trong phần này, chúng ta sẽ bổ sung các RESTful API cho các tính năng sau:</t>
+  </si>
+  <si>
+    <t>- Xem danh sách cầu thủ bóng đá.</t>
+  </si>
+  <si>
+    <t>- Xem chi tiết một cầu thủ.</t>
+  </si>
+  <si>
+    <t>- Thêm mới một cầu thủ.</t>
+  </si>
+  <si>
+    <t>- Cập nhật một cầu thủ.</t>
+  </si>
+  <si>
+    <t>Trong phần này, chúng sẽ tính hợp AJAX thông qua 2 tính năng:</t>
+  </si>
+  <si>
+    <t>1. Xây dựng chức năng danh sách cầu thủ, với dữ liệu sẽ được lấy từ Web Service thông qua Ajax.</t>
+  </si>
+  <si>
+    <t>2. Thêm mới cầu thủ, với các thông tin sẽ được truyền sang Web Service và đăng ký vào DB.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t>Lưu ý:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+      </rPr>
+      <t xml:space="preserve"> Khi thêm mới thành công thì sẽ hiển thị thông báo bởi Modal + toàn bộ thông tin sẽ clear.</t>
+    </r>
+  </si>
+  <si>
+    <t>Và trang web sẽ không bị load lại.</t>
+  </si>
+  <si>
+    <r>
       <t>Thực hiện việc sử dụng validate cho chức năng thêm mới và chỉnh sửa cầu thủ
 - Tên không được để</t>
     </r>
@@ -183,187 +359,6 @@
 - Kinh nghiệm phải là số nguyên dương
 - Vị trí phải là 1 trong các giá trị sau: trung vệ, hậu vệ, tiền vệ, tiền đạo và thủ môn</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Bài 1: Nâng cấp ứng dụng quản lý cầu thủ bóng đá </t>
-  </si>
-  <si>
-    <t>Ngoài các chức năng hiện có, ứng dụng còn cho phép tạo đội hình 11 người dựa trên danh sách cầu thủ hiện tại.</t>
-  </si>
-  <si>
-    <t>Ở màn hình danh sách cầu thủ, mặc định trạng thái của một cầu thủ là "Dự bị".</t>
-  </si>
-  <si>
-    <t>Mỗi lần cầu thủ được [Đăng ký đá] thì trạng thái cầu thủ sẽ thay đổi "Đã đăng ký".</t>
-  </si>
-  <si>
-    <t>Một cầu thủ có thể bị huỷ đăng ký, thì trạng thái sẽ được chuyển lại thành "Dự bị".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Số lượng cầu thủ đăng ký tối đã chỉ được phép là 11 người. </t>
-  </si>
-  <si>
-    <t>Thực hiện 3 chức năng sau:</t>
-  </si>
-  <si>
-    <t>1. Nếu số lượng cầu thủ đăng ký vượt quá 11 thì sẽ chuyển sang màn hình lỗi.</t>
-  </si>
-  <si>
-    <t>2. Thực hiện ghi log tất cả các hành động khiến trạng thái cầu thủ bị thay đổi.</t>
-  </si>
-  <si>
-    <t>- "Dự bị" -&gt; "Đăng ký đá".</t>
-  </si>
-  <si>
-    <t>- "Đăng ký đá" -&gt; "Dự bị".</t>
-  </si>
-  <si>
-    <t>3. Thực hiện ghi log số lượng cầu thủ được đăng ký đá.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve">Bước 1: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Chỉnh sửa màn hình danh sách cầu thủ, chuyển đổi từ table sang dạng card, như bên dưới:</t>
-    </r>
-  </si>
-  <si>
-    <t>https://getbootstrap.com/docs/5.3/components/card/#example</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve">Bước 2: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Khi người dùng click vào cầu thủ bất kì, sẽ chuyển tiếp đến trang Chi tiết cầu thủ.</t>
-    </r>
-  </si>
-  <si>
-    <t>Khi click vào button [Yêu thích], thì cầu thủ sẽ được cập nhật vào danh sách yêu thích.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Lưu ý</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>: Lưu trữ danh sách cầu thủ yêu thích vào Session.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Bước 3:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve"> Khi vào màn hình Danh sách cầu thủ yêu thích, thì sẽ hiển thị toàn bộ cầu thủ đã được Yêu thích ở Bước 2.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve">Bước 4: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Ngoài ra, cần giữ lại danh sách yêu thích khi tắt browser, sử dụng Cookie để thực hiện việc này.</t>
-    </r>
-  </si>
-  <si>
-    <t>Trong phần này, chúng ta sẽ bổ sung các RESTful API cho các tính năng sau:</t>
-  </si>
-  <si>
-    <t>- Xem danh sách cầu thủ bóng đá.</t>
-  </si>
-  <si>
-    <t>- Xem chi tiết một cầu thủ.</t>
-  </si>
-  <si>
-    <t>- Thêm mới một cầu thủ.</t>
-  </si>
-  <si>
-    <t>- Cập nhật một cầu thủ.</t>
-  </si>
-  <si>
-    <t>Trong phần này, chúng sẽ tính hợp AJAX thông qua 2 tính năng:</t>
-  </si>
-  <si>
-    <t>1. Xây dựng chức năng danh sách cầu thủ, với dữ liệu sẽ được lấy từ Web Service thông qua Ajax.</t>
-  </si>
-  <si>
-    <t>2. Thêm mới cầu thủ, với các thông tin sẽ được truyền sang Web Service và đăng ký vào DB.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Lưu ý:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve"> Khi thêm mới thành công thì sẽ hiển thị thông báo bởi Modal + toàn bộ thông tin sẽ clear.</t>
-    </r>
-  </si>
-  <si>
-    <t>Và trang web sẽ không bị load lại.</t>
   </si>
 </sst>
 </file>
@@ -706,43 +701,43 @@
     </row>
     <row r="5" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C7" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C10" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C11" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
       <c r="C12" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -771,32 +766,32 @@
     </row>
     <row r="5" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C7" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -825,12 +820,12 @@
     </row>
     <row r="5" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -841,22 +836,22 @@
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C10" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1098,9 +1093,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:20" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:20" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="8" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -1147,62 +1142,62 @@
     </row>
     <row r="5" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>